<commit_message>
chore: snapshot in-progress work on sw-config-update-batch branch
Bundles branch-relevant updates (orchestrator/commission-train SKILLs,
contracts, fleet-status, settings) together with accumulated session
scratch: morning-brief skill + dashboard, MAR5/SDD docx edits, fleet
findings JSON, and various PowerShell helper scripts.

Excludes embedded .claude/worktrees/* and the Excel lock file.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/trackers/cable-issues-tracker.xlsx
+++ b/trackers/cable-issues-tracker.xlsx
@@ -18,7 +18,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
+  </numFmts>
   <fonts count="13">
     <font>
       <name val="Calibri"/>
@@ -155,7 +158,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -209,6 +212,12 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -706,7 +715,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O105"/>
+  <dimension ref="A1:O108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -933,7 +942,7 @@
       </c>
       <c r="O3" s="3" t="inlineStr">
         <is>
-          <t>See Stadler_4736-108_Cabling_Fault_Report_v1.0.docx</t>
+          <t>See Stadler_4736-108_Cabling_Fault_Report_v1.0.docx. 2026-05-19: Confirmed active — C3 trunk swap causing STP topology churn. Switches renew DHCP every 2min but IPs constantly shift; SSH TCP SYN sent by CCU but no reply. tcpdump confirms L2 path OK (ARP works) but STP instability prevents stable management access.</t>
         </is>
       </c>
     </row>
@@ -1000,7 +1009,7 @@
       </c>
       <c r="O4" s="3" t="inlineStr">
         <is>
-          <t>See Stadler_4736-108_Cabling_Fault_Report_v1.0.docx</t>
+          <t>See Stadler_4736-108_Cabling_Fault_Report_v1.0.docx. 2026-05-19: Confirmed active — missing D1↔E2 trunk means coaches D/E are isolated from CCU. Only 5-6 of 18 switches visible at any time.</t>
         </is>
       </c>
     </row>
@@ -1072,21 +1081,69 @@
       </c>
     </row>
     <row r="6" ht="36" customHeight="1">
-      <c r="A6" s="2" t="n"/>
-      <c r="B6" s="3" t="n"/>
-      <c r="C6" s="2" t="n"/>
-      <c r="D6" s="3" t="n"/>
-      <c r="E6" s="3" t="n"/>
-      <c r="F6" s="3" t="n"/>
-      <c r="G6" s="3" t="n"/>
-      <c r="H6" s="3" t="n"/>
-      <c r="I6" s="3" t="n"/>
-      <c r="J6" s="2" t="n"/>
-      <c r="K6" s="2" t="n"/>
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>4736-104</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>6-car</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>D3</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>e1-2 (AP trunk)</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>faulty SFP/cable</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>PoE active (~2.5W class-3, device powered) but Ethernet data link never negotiates. Line DOWN, Speed/Duplex stuck Auto/Auto, no MAC learned, all error counters zero.</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>AP D4 connected to D3 e1-2 with link UP at 1G full-duplex.</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>1. Replace patch cable between AP D4 and switch D3 e1-2 (data pairs likely damaged, power pairs intact). 2. If no improvement, swap AP with known-good unit. 3. If still failing, investigate switch-side of D3 e1-2.</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="K6" s="23" t="n">
+        <v>46151</v>
+      </c>
       <c r="L6" s="2" t="n"/>
       <c r="M6" s="3" t="n"/>
-      <c r="N6" s="3" t="n"/>
-      <c r="O6" s="3" t="n"/>
+      <c r="N6" s="3" t="inlineStr">
+        <is>
+          <t>Nomad Digital</t>
+        </is>
+      </c>
+      <c r="O6" s="3" t="inlineStr">
+        <is>
+          <t>Confirmed via PoE cycle test on 2026-05-09 (box1-t10, 10.179.10.1). PoE flowing 2.5W class-3 but PHY never negotiates. 23/24 APs visible on 4736-104.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="36" customHeight="1">
       <c r="A7" s="2" t="n"/>
@@ -2770,6 +2827,201 @@
       <c r="M105" s="3" t="n"/>
       <c r="N105" s="3" t="n"/>
       <c r="O105" s="3" t="n"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B106" s="3" t="inlineStr">
+        <is>
+          <t>4734-113</t>
+        </is>
+      </c>
+      <c r="C106" s="2" t="inlineStr">
+        <is>
+          <t>6-car(?)</t>
+        </is>
+      </c>
+      <c r="D106" s="3" t="inlineStr">
+        <is>
+          <t>Unknown - 3 switches absent</t>
+        </is>
+      </c>
+      <c r="E106" s="3" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="F106" s="3" t="inlineStr">
+        <is>
+          <t>missing trunk</t>
+        </is>
+      </c>
+      <c r="G106" s="3" t="inlineStr">
+        <is>
+          <t>15 of 18 switches visible in DHCP lease table; 3 switches absent from management VLAN sweep (fping 10.179.42.128-255)</t>
+        </is>
+      </c>
+      <c r="H106" s="3" t="inlineStr">
+        <is>
+          <t>All 18 switches reachable on management VLAN</t>
+        </is>
+      </c>
+      <c r="I106" s="3" t="inlineStr">
+        <is>
+          <t>Identify which 3 cars' switch positions are missing; inspect cable/power at those switch locations. Run LLDP topology check once all switches are reachable.</t>
+        </is>
+      </c>
+      <c r="J106" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="K106" s="23" t="n">
+        <v>46161</v>
+      </c>
+      <c r="L106" s="2" t="n"/>
+      <c r="M106" s="3" t="n"/>
+      <c r="N106" s="3" t="inlineStr">
+        <is>
+          <t>Nomad Digital</t>
+        </is>
+      </c>
+      <c r="O106" s="3" t="inlineStr">
+        <is>
+          <t>Detected 2026-05-19 via CCU 10.179.42.1 DHCP lease scan. Only 15 leases with VDS OUI a0:59:3a. May indicate 3 switches without power or with cable fault at inter-coach trunk or management port.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B107" s="3" t="inlineStr">
+        <is>
+          <t>4734-109</t>
+        </is>
+      </c>
+      <c r="C107" s="2" t="inlineStr">
+        <is>
+          <t>4-car</t>
+        </is>
+      </c>
+      <c r="D107" s="3" t="inlineStr">
+        <is>
+          <t>B1 / B3 - ZFR access port</t>
+        </is>
+      </c>
+      <c r="E107" s="3" t="inlineStr">
+        <is>
+          <t>B1 e1-11 / B3 e1-11</t>
+        </is>
+      </c>
+      <c r="F107" s="3" t="inlineStr">
+        <is>
+          <t>AP not connected</t>
+        </is>
+      </c>
+      <c r="G107" s="3" t="inlineStr">
+        <is>
+          <t>Both ZFR access ports (B1 e1-11, B3 e1-11) admin-enabled but link DOWN; no ZFR device responding</t>
+        </is>
+      </c>
+      <c r="H107" s="3" t="inlineStr">
+        <is>
+          <t>B1 e1-11 and B3 e1-11 UP at 1G with ZFR device connected (VLAN 2 access port)</t>
+        </is>
+      </c>
+      <c r="I107" s="3" t="inlineStr">
+        <is>
+          <t>Verify ZFR devices are physically installed and powered at B1 and B3 positions on Fzg 9. Check patch cable from switch port to ZFR unit.</t>
+        </is>
+      </c>
+      <c r="J107" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="K107" s="23" t="n">
+        <v>46161</v>
+      </c>
+      <c r="L107" s="2" t="n"/>
+      <c r="M107" s="3" t="n"/>
+      <c r="N107" s="3" t="inlineStr">
+        <is>
+          <t>Nomad Digital</t>
+        </is>
+      </c>
+      <c r="O107" s="3" t="inlineStr">
+        <is>
+          <t>Detected 2026-05-19 via CCU 10.179.38.1. show interface B1.e1-11 and B3.e1-11: admin enabled, line protocol down. Switch config v5. FW: ARP at 172.19.132.129 (Westermo default .129 = uncommissioned).</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B108" s="3" t="inlineStr">
+        <is>
+          <t>4734-112</t>
+        </is>
+      </c>
+      <c r="C108" s="2" t="inlineStr">
+        <is>
+          <t>5-car</t>
+        </is>
+      </c>
+      <c r="D108" s="3" t="inlineStr">
+        <is>
+          <t>C3 - all 4x10G ports UP</t>
+        </is>
+      </c>
+      <c r="E108" s="3" t="inlineStr">
+        <is>
+          <t>C3 e0-0/e0-1/e0-2/e0-3</t>
+        </is>
+      </c>
+      <c r="F108" s="3" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="G108" s="3" t="inlineStr">
+        <is>
+          <t>C3 switch has 4x10G ports all UP simultaneously - unusual for a non-end-junction switch in a 5-car consist; expected topology only requires 2 inter-coach trunks</t>
+        </is>
+      </c>
+      <c r="H108" s="3" t="inlineStr">
+        <is>
+          <t>C3 should have 2 active inter-coach trunks (e0-0 and e0-1); e0-2/e0-3 role unclear without schema for 4734-112</t>
+        </is>
+      </c>
+      <c r="I108" s="3" t="inlineStr">
+        <is>
+          <t>Run LLDP topology check on C3 (CCU 10.179.41.1) to identify all 4 peer switch identities. Cross-reference against 4734-112 IP-allocation schema PDF to confirm if e0-2/e0-3 carry a valid purpose or are anomalous.</t>
+        </is>
+      </c>
+      <c r="J108" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="K108" s="23" t="n">
+        <v>46161</v>
+      </c>
+      <c r="L108" s="2" t="n"/>
+      <c r="M108" s="3" t="n"/>
+      <c r="N108" s="3" t="inlineStr">
+        <is>
+          <t>Nomad Digital</t>
+        </is>
+      </c>
+      <c r="O108" s="3" t="inlineStr">
+        <is>
+          <t>Detected 2026-05-19. Train is 5-car (A,B,C,E,F cars - 15 switches, 20 APs per DHCP). vlan7 was misconfigured (172.19.243.130 stale); fixed to 172.19.134.2/17 and persisted via chroot on 2026-05-19. Switch config v3. C3 anomaly needs schema verification.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="J2:J105">

</xml_diff>